<commit_message>
La Primavera Race 1
</commit_message>
<xml_diff>
--- a/SpringClassics/SpringClassics.xlsx
+++ b/SpringClassics/SpringClassics.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ride the White Roads race 1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ride the White Roads race 2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="La Primavera race 1" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1789,7 +1790,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Team Not Pogi</t>
+          <t>SISU Racing</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -3009,6 +3010,663 @@
       </c>
       <c r="I39" t="n">
         <v>2.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>pen</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>zwift_id</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>team_name</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>avg_power</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>avg_wkg</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>182292</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>JOHAN GREN</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>eSRT</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>01:15:14.388</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>328</v>
+      </c>
+      <c r="I2" t="n">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1417072</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Kelvin Newman</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>teamWKG</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>01:16:14.454</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>60.066</v>
+      </c>
+      <c r="H3" t="n">
+        <v>246</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1175748</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Jos Castelijns(TeamNL)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TeamNL</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>01:16:14.679</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>60.291</v>
+      </c>
+      <c r="H4" t="n">
+        <v>300</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3102903</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>&amp;#321;ukasz Dul</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>T175</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>01:17:07.587</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>113.199</v>
+      </c>
+      <c r="H5" t="n">
+        <v>284</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1593779</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Alberto Goldoni (TSE)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>TSE</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>01:21:22.240</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>367.852</v>
+      </c>
+      <c r="H6" t="n">
+        <v>291</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1387591</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Tommy Sellars (TFC Typhoon)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>TFC</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>01:23:31.337</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>496.949</v>
+      </c>
+      <c r="H7" t="n">
+        <v>296</v>
+      </c>
+      <c r="I7" t="n">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>3640893</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Christian Strauch</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>01:23:54.202</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>519.814</v>
+      </c>
+      <c r="H8" t="n">
+        <v>253</v>
+      </c>
+      <c r="I8" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>3353670</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Wim Van Cutsem [BikeRepublic]</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BikeRepublic</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>01:23:56.168</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>247</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1948296</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jorge Sanchis </t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>01:28:21.240</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>221</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>8086912</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R G Cycling  (Diabetic Cyclist) </t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>01:29:59.274</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>98.03400000000001</v>
+      </c>
+      <c r="H11" t="n">
+        <v>181</v>
+      </c>
+      <c r="I11" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>6345533</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Mark Tighe</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>INOX</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>01:36:40.454</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>499.214</v>
+      </c>
+      <c r="H12" t="n">
+        <v>195</v>
+      </c>
+      <c r="I12" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>6411187</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Ken Wahid</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>01:32:47.373</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>202</v>
+      </c>
+      <c r="I13" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>6147623</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>John Moulding</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>01:36:40.302</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>232.929</v>
+      </c>
+      <c r="H14" t="n">
+        <v>207</v>
+      </c>
+      <c r="I14" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>229572</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fabio Bevilacqua (TDRS) </t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Team Italy</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>01:36:51.461</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>244.088</v>
+      </c>
+      <c r="H15" t="n">
+        <v>177</v>
+      </c>
+      <c r="I15" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>3622652</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Francky Lootvoet</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>01:37:22.310</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>274.937</v>
+      </c>
+      <c r="H16" t="n">
+        <v>187</v>
+      </c>
+      <c r="I16" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>7669986</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Ren&amp;eacute; Servais</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>01:43:24.788</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>183</v>
+      </c>
+      <c r="I17" t="n">
+        <v>2.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>